<commit_message>
date fix, filters fix
</commit_message>
<xml_diff>
--- a/bams-backend/app/ds/llm/utils/Bank Accounts V1.xlsx
+++ b/bams-backend/app/ds/llm/utils/Bank Accounts V1.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="75">
   <si>
     <t>S No</t>
   </si>
@@ -202,7 +202,7 @@
     <t>MODERN FLOUR MILLS PVT LTD</t>
   </si>
   <si>
-    <t>CURRENT ACCOUNT FOR MCA</t>
+    <t>Current</t>
   </si>
   <si>
     <t>MODE478003676</t>
@@ -211,10 +211,7 @@
     <t>Business</t>
   </si>
   <si>
-    <t>Catterpillar Realty Spaces Pvt. Ltd.</t>
-  </si>
-  <si>
-    <t>Current Account</t>
+    <t>Caterpillar Realty Spaces Pvt. Ltd.</t>
   </si>
   <si>
     <t>Goldstone Realty Ventures Pvt. Ltd.</t>
@@ -689,7 +686,7 @@
   <cols>
     <col min="1" max="1" width="21.142857142857142" customWidth="1"/>
     <col min="2" max="2" width="36.714285714285715" customWidth="1"/>
-    <col min="3" max="3" width="13.571428571428571" customWidth="1"/>
+    <col min="3" max="3" width="50.42857142857143" customWidth="1"/>
     <col min="4" max="4" width="34.142857142857146" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="17.714285714285715" customWidth="1"/>
@@ -1851,7 +1848,7 @@
         <v>66</v>
       </c>
       <c r="C48" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D48">
         <v>99919871207208</v>
@@ -1868,10 +1865,10 @@
         <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C49" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D49">
         <v>99929871207208</v>
@@ -1885,13 +1882,13 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>68</v>
+      </c>
+      <c r="B50" t="s">
         <v>69</v>
       </c>
-      <c r="B50" t="s">
-        <v>70</v>
-      </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D50">
         <v>20100079871280</v>
@@ -1905,10 +1902,10 @@
         <v>54</v>
       </c>
       <c r="B51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C51" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D51">
         <v>99909871207208</v>
@@ -1925,10 +1922,10 @@
         <v>8</v>
       </c>
       <c r="B52" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C52" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D52">
         <v>478010200005432</v>
@@ -1939,13 +1936,13 @@
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>72</v>
+      </c>
+      <c r="B53" t="s">
         <v>73</v>
       </c>
-      <c r="B53" t="s">
-        <v>74</v>
-      </c>
       <c r="C53" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D53">
         <v>201003501000</v>
@@ -1956,13 +1953,13 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B54" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C54" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D54">
         <v>201003427577</v>

</xml_diff>